<commit_message>
Added resistor values for window comparator threshold dividers to sensor excel
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/rbad163_uoa_auckland_ac_nz/Documents/University/Engineering/Stage 3/Semester 2/ELECTENG 311/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="682" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8C97358-58A2-40C7-9ECB-B330F5D84607}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72C987A-9FDB-4982-8A43-87E8D8215585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
     <sheet name="Temp Sensor" sheetId="2" r:id="rId2"/>
     <sheet name="Voltage Sensor" sheetId="4" r:id="rId3"/>
     <sheet name="Window Comparator" sheetId="6" r:id="rId4"/>
+    <sheet name="Reference Voltage" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="82">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -251,7 +252,43 @@
     <t>Vcc / (R_temp_high + R1)</t>
   </si>
   <si>
-    <t>Note: Graph generated from window_comparator LTSpice file</t>
+    <t>V_THH</t>
+  </si>
+  <si>
+    <t>Current Sensor</t>
+  </si>
+  <si>
+    <t>Voltage Sensor</t>
+  </si>
+  <si>
+    <t>Temperature Sensor</t>
+  </si>
+  <si>
+    <t>V_THL</t>
+  </si>
+  <si>
+    <t>Theoretical</t>
+  </si>
+  <si>
+    <t>Pratical</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>8.2 kΩ</t>
+  </si>
+  <si>
+    <t>47 KΩ</t>
+  </si>
+  <si>
+    <t>22 kΩ</t>
+  </si>
+  <si>
+    <t>47 kΩ</t>
+  </si>
+  <si>
+    <t>5.6 kΩ</t>
   </si>
 </sst>
 </file>
@@ -262,7 +299,7 @@
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -340,6 +377,13 @@
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -369,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -413,20 +457,23 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,115 +651,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE2F21D7-3F0A-9F11-F04D-DE5F031DDCCF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2914650" y="1981200"/>
-          <a:ext cx="11087100" cy="7658100"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>50</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 11">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{470BA941-AAA4-062D-D3F9-3403EDB2515A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14820900" y="1981200"/>
-          <a:ext cx="19183350" cy="10039350"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -750,7 +692,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -856,7 +798,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -998,7 +940,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1007,26 +949,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:Q14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="67.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="38.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" style="2" customWidth="1"/>
-    <col min="5" max="7" width="9.140625" style="2"/>
-    <col min="8" max="9" width="38.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" style="2" customWidth="1"/>
-    <col min="11" max="13" width="9.140625" style="2"/>
-    <col min="14" max="14" width="47.7109375" style="2" customWidth="1"/>
-    <col min="15" max="15" width="76.140625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="18.7109375" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="40.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="67.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="38.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" style="2" customWidth="1"/>
+    <col min="5" max="7" width="9.109375" style="2"/>
+    <col min="8" max="9" width="38.6640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="2" customWidth="1"/>
+    <col min="11" max="13" width="9.109375" style="2"/>
+    <col min="14" max="14" width="47.6640625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="76.109375" style="2" customWidth="1"/>
+    <col min="16" max="16" width="18.6640625" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="7"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -1050,7 +992,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="35.25" customHeight="1">
+    <row r="3" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1062,27 +1004,27 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="73.5" customHeight="1">
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
+    <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="N4" s="16" t="s">
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="N4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-    </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1">
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+    </row>
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
@@ -1122,7 +1064,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1164,7 +1106,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
@@ -1206,7 +1148,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>24</v>
       </c>
@@ -1248,7 +1190,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1290,7 +1232,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
@@ -1319,7 +1261,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1">
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1338,7 +1280,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="35.25" customHeight="1">
+    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -1357,7 +1299,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="35.25" customHeight="1">
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H13" s="1" t="s">
         <v>43</v>
       </c>
@@ -1372,7 +1314,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="35.25" customHeight="1">
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H14" s="2" t="s">
         <v>45</v>
       </c>
@@ -1401,28 +1343,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F2E2C88-472F-40E6-9BB7-0CE3D1C9A840}">
   <dimension ref="B1:Q10"/>
-  <sheetFormatPr defaultRowHeight="35.25" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="58.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
-    <col min="6" max="7" width="9.140625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="34.42578125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="40.85546875" style="5" customWidth="1"/>
-    <col min="10" max="10" width="25.42578125" style="5" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" style="5" customWidth="1"/>
-    <col min="12" max="13" width="9.140625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="34.42578125" style="5" customWidth="1"/>
-    <col min="15" max="15" width="52.85546875" style="5" customWidth="1"/>
-    <col min="16" max="16" width="17.5703125" style="5" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="5" customWidth="1"/>
-    <col min="18" max="16380" width="9.140625" style="5" customWidth="1"/>
-    <col min="16381" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="7" width="9.109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="34.44140625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="40.88671875" style="5" customWidth="1"/>
+    <col min="10" max="10" width="25.44140625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" style="5" customWidth="1"/>
+    <col min="12" max="13" width="9.109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="34.44140625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="52.88671875" style="5" customWidth="1"/>
+    <col min="16" max="16" width="17.5546875" style="5" customWidth="1"/>
+    <col min="17" max="17" width="9.6640625" style="5" customWidth="1"/>
+    <col min="18" max="16380" width="9.109375" style="5" customWidth="1"/>
+    <col min="16381" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1440,7 +1382,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="57.75" customHeight="1">
+    <row r="2" spans="2:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>47</v>
       </c>
@@ -1466,7 +1408,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>6</v>
       </c>
@@ -1508,7 +1450,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="69.75" customHeight="1">
+    <row r="5" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>51</v>
       </c>
@@ -1552,7 +1494,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="69.75" customHeight="1">
+    <row r="6" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>56</v>
       </c>
@@ -1596,7 +1538,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>62</v>
       </c>
@@ -1631,7 +1573,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>66</v>
       </c>
@@ -1666,7 +1608,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1684,7 +1626,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1711,13 +1653,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD44C968-61FF-4F4E-9D6C-A1C9337DEECD}">
   <dimension ref="B1:Q8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1735,7 +1677,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10"/>
       <c r="C2" s="12"/>
       <c r="D2" s="1"/>
@@ -1753,7 +1695,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
@@ -1771,7 +1713,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1789,7 +1731,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -1807,7 +1749,7 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1825,7 +1767,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -1851,96 +1793,118 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC3F59B-30C5-40B9-A90E-89A9AC3DA184}">
-  <dimension ref="B1:S8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1"/>
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="20" width="16.77734375" style="5" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:19" ht="150" customHeight="1">
-      <c r="B1" s="19" t="s">
+    <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+    </row>
+    <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G2" s="15"/>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
-    </row>
-    <row r="2" spans="2:19" ht="35.25" customHeight="1">
-      <c r="B2" s="10"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-    </row>
-    <row r="4" spans="2:19" ht="35.25" customHeight="1">
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+      <c r="C3" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="1">
+        <v>4.25</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="D4" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="F4" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0.5</v>
+      </c>
       <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="1"/>
-    </row>
-    <row r="5" spans="2:19" ht="35.25" customHeight="1">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
+    </row>
+    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="1">
+        <v>4.2569999999999997</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.74299999999999999</v>
+      </c>
+      <c r="D5" s="1">
+        <v>3.4060000000000001</v>
+      </c>
+      <c r="E5" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="F5" s="1">
+        <v>4.468</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0.53200000000000003</v>
+      </c>
       <c r="H5" s="1"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-    </row>
-    <row r="6" spans="2:19" ht="35.25" customHeight="1">
+    </row>
+    <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -1948,8 +1912,6 @@
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="13"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -1960,7 +1922,7 @@
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
     </row>
-    <row r="7" spans="2:19" ht="35.25" customHeight="1">
+    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1980,19 +1942,25 @@
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
     </row>
-    <row r="8" spans="2:19" ht="35.25" customHeight="1">
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
+    <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -2000,12 +1968,137 @@
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
     </row>
+    <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="M9" s="15"/>
+    </row>
+    <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="K11" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:S1"/>
+  <mergeCells count="12">
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="J8:M8"/>
   </mergeCells>
+  <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F0E4DC-8390-40EC-853B-5309BBADFFFF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added window comparator diagrams to sensor excel
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72C987A-9FDB-4982-8A43-87E8D8215585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46494A56-1F19-4CD4-9C0F-A1BA4A224E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -651,6 +651,111 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>923925</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>285750</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{519287D1-16A4-5F20-3B3C-FC30B969B3E6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2914650" y="6819900"/>
+          <a:ext cx="13363575" cy="7639050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>435750</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>16650</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>559575</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>226200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F5A5C0B-A9EE-BF20-75EF-01EF3DC68E85}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16933050" y="9808350"/>
+          <a:ext cx="4695825" cy="4591050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -2090,6 +2195,7 @@
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Updated sensor excel graphs
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46494A56-1F19-4CD4-9C0F-A1BA4A224E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCE060AC-2046-49C8-A99C-B5F0FB85811E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Temp Sensor" sheetId="2" r:id="rId2"/>
     <sheet name="Voltage Sensor" sheetId="4" r:id="rId3"/>
     <sheet name="Window Comparator" sheetId="6" r:id="rId4"/>
-    <sheet name="Reference Voltage" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="88">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -285,10 +284,28 @@
     <t>22 kΩ</t>
   </si>
   <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
     <t>47 kΩ</t>
   </si>
   <si>
     <t>5.6 kΩ</t>
+  </si>
+  <si>
+    <t>R5</t>
+  </si>
+  <si>
+    <t>R6</t>
+  </si>
+  <si>
+    <t>470 k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Threshold Hysteresis = 100 mV </t>
   </si>
 </sst>
 </file>
@@ -497,22 +514,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>60975</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>127523</xdr:rowOff>
+      <xdr:colOff>115957</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>82826</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>546653</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>443361</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1900446</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>442706</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A95F0D3-95D3-11F4-9EB0-F0A28BEFB918}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A2BF54B4-1D4F-FF5B-3E81-3D8E6F752292}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -534,8 +551,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2711410" y="6670784"/>
-          <a:ext cx="10292286" cy="6577490"/>
+          <a:off x="2898914" y="8282609"/>
+          <a:ext cx="12220575" cy="8410575"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -601,22 +618,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
+      <xdr:colOff>152400</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>473529</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>212271</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>342900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{24A2B483-C3D2-294B-A553-73E9C6638DC6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82D2BA0D-E552-94DB-183E-D5D84D3E6E44}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -638,8 +655,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="696686" y="522514"/>
-          <a:ext cx="10325100" cy="7277100"/>
+          <a:off x="2933700" y="2000250"/>
+          <a:ext cx="11449050" cy="5943600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -653,56 +670,6 @@
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>923925</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{519287D1-16A4-5F20-3B3C-FC30B969B3E6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2914650" y="6819900"/>
-          <a:ext cx="13363575" cy="7639050"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>13</xdr:col>
@@ -730,7 +697,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -745,6 +712,56 @@
         <a:xfrm>
           <a:off x="16933050" y="9808350"/>
           <a:ext cx="4695825" cy="4591050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>962025</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>266700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2F28B648-1910-0276-5D8B-E83709E2AA67}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2952750" y="6800850"/>
+          <a:ext cx="13363575" cy="7639050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1940,6 +1957,12 @@
       </c>
       <c r="G2" s="15"/>
       <c r="H2" s="10"/>
+      <c r="I2" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
     </row>
     <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="10" t="s">
@@ -1960,6 +1983,14 @@
       <c r="G3" s="10" t="s">
         <v>73</v>
       </c>
+      <c r="I3" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="L3" s="15"/>
     </row>
     <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -1984,6 +2015,18 @@
         <v>0.5</v>
       </c>
       <c r="H4" s="10"/>
+      <c r="I4" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -2008,6 +2051,18 @@
         <v>0.53200000000000003</v>
       </c>
       <c r="H5" s="1"/>
+      <c r="I5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
@@ -2148,7 +2203,7 @@
         <v>78</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>77</v>
@@ -2157,31 +2212,34 @@
         <v>79</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="15">
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="L9:M9"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="D9:E9"/>
@@ -2199,15 +2257,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F0E4DC-8390-40EC-853B-5309BBADFFFF}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{b75eb9d1-7479-4f8a-9240-cc5b19dbbc64}" enabled="1" method="Standard" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="0"/>

</xml_diff>

<commit_message>
Added anti-aliasing filer sheet to sensor excel
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCE060AC-2046-49C8-A99C-B5F0FB85811E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC26DCB-1044-4358-9710-6DE7E9DB7E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="Temp Sensor" sheetId="2" r:id="rId2"/>
     <sheet name="Voltage Sensor" sheetId="4" r:id="rId3"/>
     <sheet name="Window Comparator" sheetId="6" r:id="rId4"/>
+    <sheet name="Anti-Aliasing Filter" sheetId="9" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="96">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -306,6 +307,30 @@
   </si>
   <si>
     <t xml:space="preserve">Threshold Hysteresis = 100 mV </t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>1 / 2 *pi * R1 * f_cutoff</t>
+  </si>
+  <si>
+    <t>f_sample</t>
+  </si>
+  <si>
+    <t>Hz</t>
+  </si>
+  <si>
+    <t>For an ADC clock of 200 kHz, at 13 cycles per sample</t>
+  </si>
+  <si>
+    <t>f_cutoff</t>
+  </si>
+  <si>
+    <t>f_sample / 2</t>
+  </si>
+  <si>
+    <t>F</t>
   </si>
 </sst>
 </file>
@@ -514,22 +539,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>115957</xdr:colOff>
+      <xdr:colOff>82826</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>82826</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1900446</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>442706</xdr:rowOff>
+      <xdr:colOff>1867315</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>4556</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A2BF54B4-1D4F-FF5B-3E81-3D8E6F752292}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95B386D9-2BD7-471E-5C49-9D7ED902899C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -551,7 +576,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2898914" y="8282609"/>
+          <a:off x="2865783" y="8282609"/>
           <a:ext cx="12220575" cy="8410575"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -569,71 +594,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>85725</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>560614</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>428625</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{83434D82-0F20-D811-27E7-AE4F696DF7CC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2800350" y="8572500"/>
-          <a:ext cx="9075964" cy="8801100"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>342900</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1790700</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82D2BA0D-E552-94DB-183E-D5D84D3E6E44}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12C36A2F-BE78-B6F1-8A67-F7B46D62FAEB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -655,7 +631,62 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2933700" y="2000250"/>
+          <a:off x="2895600" y="6572250"/>
+          <a:ext cx="11144250" cy="5734050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>285750</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B454C22-703E-E42A-236D-E42CA9732861}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2819400" y="1943100"/>
           <a:ext cx="11449050" cy="5943600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -762,6 +793,61 @@
         <a:xfrm>
           <a:off x="2952750" y="6800850"/>
           <a:ext cx="13363575" cy="7639050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>361950</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD31F69F-F3AE-7C2D-8AA9-21DAEFDE15BA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11315700" y="2000250"/>
+          <a:ext cx="6972300" cy="3829050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1761,10 +1847,18 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
+      <c r="N10" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="O10" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P10" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q10" s="10" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2257,6 +2351,199 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DDA2E54-9BDB-4BF6-80B7-49457B01E1DD}">
+  <dimension ref="B1:Q8"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+    </row>
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+    </row>
+    <row r="3" spans="2:17" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="5">
+        <v>16000</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="5">
+        <f>D3 / 2</f>
+        <v>8000</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+    </row>
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="5">
+        <v>4700</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="1">
+        <f>1 / (2 * PI() * D5 *D4)</f>
+        <v>4.232844231167429E-9</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{b75eb9d1-7479-4f8a-9240-cc5b19dbbc64}" enabled="1" method="Standard" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="0"/>

</xml_diff>

<commit_message>
Minor change to sensor excel
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC26DCB-1044-4358-9710-6DE7E9DB7E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58173807-0623-440E-AC11-3349AC02C77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="96">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -1847,18 +1847,10 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="P10" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>9</v>
-      </c>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added touch sensor oscillator sheet to sensor excel
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58173807-0623-440E-AC11-3349AC02C77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21F84EB-DFAF-494E-886A-450862ED994E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Voltage Sensor" sheetId="4" r:id="rId3"/>
     <sheet name="Window Comparator" sheetId="6" r:id="rId4"/>
     <sheet name="Anti-Aliasing Filter" sheetId="9" r:id="rId5"/>
+    <sheet name="Touch Sensor Oscillator" sheetId="11" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="98">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -331,6 +332,12 @@
   </si>
   <si>
     <t>F</t>
+  </si>
+  <si>
+    <t>C_touch_sensor</t>
+  </si>
+  <si>
+    <t>Test value for simulations</t>
   </si>
 </sst>
 </file>
@@ -455,7 +462,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -516,6 +523,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -859,6 +869,61 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>110836</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1898073</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>510886</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>229466</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75FF338C-212C-9281-FBE3-BEBD0665B0A9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11388436" y="1898073"/>
+          <a:ext cx="7258050" cy="6505575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -2451,7 +2516,7 @@
       <c r="D5" s="5">
         <v>4700</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="1" t="s">
         <v>36</v>
       </c>
       <c r="F5" s="1"/>
@@ -2536,6 +2601,197 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBF5C97-B701-49E8-8D17-B57E480030E6}">
+  <dimension ref="B1:Q8"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+    </row>
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+    </row>
+    <row r="3" spans="2:17" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9">
+        <v>10000</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1">
+        <v>47000</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+    </row>
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="21">
+        <v>10000</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="21">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{b75eb9d1-7479-4f8a-9240-cc5b19dbbc64}" enabled="1" method="Standard" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="0"/>

</xml_diff>

<commit_message>
Added ground symbol to anti-aliasing filter diagram in sensor excel
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21F84EB-DFAF-494E-886A-450862ED994E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35946E6-0E9C-4E36-9C30-D1AE339D86FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="102">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -338,6 +338,18 @@
   </si>
   <si>
     <t>Test value for simulations</t>
+  </si>
+  <si>
+    <t>Vv_min</t>
+  </si>
+  <si>
+    <t>Minimum super cap voltage</t>
+  </si>
+  <si>
+    <t>Vv_max</t>
+  </si>
+  <si>
+    <t>Maximum super cap voltage</t>
   </si>
 </sst>
 </file>
@@ -507,6 +519,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -522,9 +537,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -659,15 +671,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>171450</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>285750</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>342900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -696,7 +708,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2819400" y="1943100"/>
+          <a:off x="2838450" y="5067300"/>
           <a:ext cx="11449050" cy="5943600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -714,15 +726,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>435750</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>16650</xdr:rowOff>
+      <xdr:colOff>73800</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>92850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>559575</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>226200</xdr:rowOff>
+      <xdr:colOff>197625</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>302400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -751,7 +763,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16933050" y="9808350"/>
+          <a:off x="16571100" y="6817500"/>
           <a:ext cx="4695825" cy="4591050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -819,22 +831,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
+      <xdr:colOff>27709</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:rowOff>55418</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:colOff>132484</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>361950</xdr:rowOff>
+      <xdr:rowOff>282286</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD31F69F-F3AE-7C2D-8AA9-21DAEFDE15BA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA09BFFD-8358-3974-9E54-9931187A535D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -856,8 +868,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11315700" y="2000250"/>
-          <a:ext cx="6972300" cy="3829050"/>
+          <a:off x="11305309" y="1967345"/>
+          <a:ext cx="6962775" cy="3829050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1278,24 +1290,24 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="18" t="s">
+      <c r="H4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="N4" s="17" t="s">
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="N4" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
     </row>
     <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="10" t="s">
@@ -1929,7 +1941,11 @@
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="16384" width="9.109375" style="5"/>
+    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
@@ -1951,10 +1967,18 @@
       <c r="Q1" s="1"/>
     </row>
     <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="10"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="B2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>9</v>
+      </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="10"/>
@@ -1968,11 +1992,33 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
+    <row r="3" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="10"/>
@@ -2075,45 +2121,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
+      <c r="S1" s="15"/>
     </row>
     <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15" t="s">
+      <c r="E2" s="21"/>
+      <c r="F2" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="15"/>
+      <c r="G2" s="21"/>
       <c r="H2" s="10"/>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="10" t="s">
@@ -2134,14 +2180,14 @@
       <c r="G3" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15" t="s">
+      <c r="J3" s="21"/>
+      <c r="K3" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="L3" s="15"/>
+      <c r="L3" s="21"/>
     </row>
     <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -2254,24 +2300,24 @@
       <c r="S7" s="1"/>
     </row>
     <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15" t="s">
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15" t="s">
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="21"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -2280,30 +2326,30 @@
       <c r="S8" s="1"/>
     </row>
     <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15" t="s">
+      <c r="C9" s="21"/>
+      <c r="D9" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15" t="s">
+      <c r="E9" s="21"/>
+      <c r="F9" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15" t="s">
+      <c r="G9" s="21"/>
+      <c r="H9" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15" t="s">
+      <c r="I9" s="21"/>
+      <c r="J9" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15" t="s">
+      <c r="K9" s="21"/>
+      <c r="L9" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="M9" s="15"/>
+      <c r="M9" s="21"/>
     </row>
     <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
@@ -2386,21 +2432,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="J8:M8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="H9:I9"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2699,7 +2745,7 @@
         <v>80</v>
       </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="21">
+      <c r="D5" s="16">
         <v>10000</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -2749,7 +2795,7 @@
       <c r="C7" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="16">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="E7" s="6" t="s">

</xml_diff>

<commit_message>
Added effects of practical voltage references to smarts spreadsheet
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/ctra157_uoa_auckland_ac_nz/Documents/Documents/GitHub/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35946E6-0E9C-4E36-9C30-D1AE339D86FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{F35946E6-0E9C-4E36-9C30-D1AE339D86FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66C118AF-E92A-435A-AB54-0F63D7562F70}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
@@ -43,8 +43,100 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>ctra157</author>
+  </authors>
+  <commentList>
+    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{A8C3D8B6-DE33-455B-B275-8AD8B41344DB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>ctra157:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+E12, E6, etc.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>ctra157</author>
+  </authors>
+  <commentList>
+    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{221E7002-277B-4444-82F3-0C45745BDF2C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>ctra157:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Assumes R1=R2.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0" xr:uid="{05951897-3565-4077-B2AF-9907F205D955}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>ctra157:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Assumes R1=R2.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="118">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -277,27 +369,12 @@
     <t>R2</t>
   </si>
   <si>
-    <t>8.2 kΩ</t>
-  </si>
-  <si>
-    <t>47 KΩ</t>
-  </si>
-  <si>
-    <t>22 kΩ</t>
-  </si>
-  <si>
     <t>R3</t>
   </si>
   <si>
     <t>R4</t>
   </si>
   <si>
-    <t>47 kΩ</t>
-  </si>
-  <si>
-    <t>5.6 kΩ</t>
-  </si>
-  <si>
     <t>R5</t>
   </si>
   <si>
@@ -334,9 +411,6 @@
     <t>F</t>
   </si>
   <si>
-    <t>C_touch_sensor</t>
-  </si>
-  <si>
     <t>Test value for simulations</t>
   </si>
   <si>
@@ -350,17 +424,124 @@
   </si>
   <si>
     <t>Maximum super cap voltage</t>
+  </si>
+  <si>
+    <t>Chosen Parameters</t>
+  </si>
+  <si>
+    <t>1 / (2*pi*R1*C1)</t>
+  </si>
+  <si>
+    <t>(kΩ)</t>
+  </si>
+  <si>
+    <t>Min (A)</t>
+  </si>
+  <si>
+    <t>Max (A)</t>
+  </si>
+  <si>
+    <t>Min (V)</t>
+  </si>
+  <si>
+    <t>Max (V)</t>
+  </si>
+  <si>
+    <t>Min (Ω)</t>
+  </si>
+  <si>
+    <t>Max (Ω)</t>
+  </si>
+  <si>
+    <r>
+      <t>Max (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="18"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>°</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="18"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>C)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Min (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="18"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>°</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="18"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>C)</t>
+    </r>
+  </si>
+  <si>
+    <t>(approximated from datasheet)</t>
+  </si>
+  <si>
+    <t>C_touch_sensor (no touch)</t>
+  </si>
+  <si>
+    <t>C_touch_sensor (yes touch)</t>
+  </si>
+  <si>
+    <t>f_0 (no touch)</t>
+  </si>
+  <si>
+    <t>f_0 (yes touch)</t>
+  </si>
+  <si>
+    <t>1 / (-2 * ln(1/3) * R3 * C)</t>
+  </si>
+  <si>
+    <t>T/C frequency</t>
+  </si>
+  <si>
+    <t>no. clock cycles (no touch)</t>
+  </si>
+  <si>
+    <t>no. clock cycles (yes touch)</t>
+  </si>
+  <si>
+    <t>2 MHz / 1</t>
+  </si>
+  <si>
+    <t>TC frequency / f_0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -447,6 +628,44 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -474,7 +693,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -539,6 +758,27 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -560,16 +800,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>82826</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1450964</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>82826</xdr:rowOff>
+      <xdr:rowOff>307963</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1867315</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>4556</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>103910</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>443627</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -598,8 +838,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2865783" y="8282609"/>
-          <a:ext cx="12220575" cy="8410575"/>
+          <a:off x="1450964" y="8551418"/>
+          <a:ext cx="9684628" cy="6889754"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -725,15 +965,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>73800</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>359550</xdr:colOff>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>92850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>197625</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>7125</xdr:colOff>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>302400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -763,8 +1003,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16571100" y="6817500"/>
-          <a:ext cx="4695825" cy="4591050"/>
+          <a:off x="31149113" y="1997850"/>
+          <a:ext cx="4600575" cy="4733925"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -775,16 +1015,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>171450</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>962025</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>266700</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>128588</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>266699</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -813,8 +1053,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2952750" y="6800850"/>
-          <a:ext cx="13363575" cy="7639050"/>
+          <a:off x="17816513" y="1981200"/>
+          <a:ext cx="13101638" cy="7881937"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1234,26 +1474,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:Q14"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="67.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="38.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" style="2" customWidth="1"/>
-    <col min="5" max="7" width="9.109375" style="2"/>
-    <col min="8" max="9" width="38.6640625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.6640625" style="2" customWidth="1"/>
-    <col min="11" max="13" width="9.109375" style="2"/>
-    <col min="14" max="14" width="47.6640625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="76.109375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="18.6640625" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="1" width="40.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="67.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="38.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="2" customWidth="1"/>
+    <col min="5" max="7" width="9.140625" style="2"/>
+    <col min="8" max="9" width="38.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="2" customWidth="1"/>
+    <col min="11" max="13" width="9.140625" style="2"/>
+    <col min="14" max="14" width="47.7109375" style="2" customWidth="1"/>
+    <col min="15" max="15" width="76.140625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="18.7109375" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="7"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -1277,7 +1517,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1289,7 +1529,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
       <c r="D4" s="17"/>
@@ -1309,7 +1549,7 @@
       <c r="P4" s="18"/>
       <c r="Q4" s="18"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
@@ -1349,7 +1589,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1372,7 +1612,7 @@
       </c>
       <c r="J6" s="1">
         <f>D7*D10</f>
-        <v>-1.7500000000000002E-2</v>
+        <v>-1.7000000000000001E-2</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>12</v>
@@ -1385,13 +1625,13 @@
       </c>
       <c r="P6" s="2">
         <f>POWER(D7,2)*D10</f>
-        <v>3.0624999999999999E-2</v>
+        <v>4.2500000000000003E-3</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
@@ -1399,7 +1639,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="1">
-        <v>-1.75</v>
+        <v>-0.25</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>19</v>
@@ -1414,7 +1654,7 @@
       </c>
       <c r="J7" s="1">
         <f>D8*D10</f>
-        <v>1.7500000000000002E-2</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>12</v>
@@ -1427,13 +1667,13 @@
       </c>
       <c r="P7" s="2">
         <f>POWER(D8,2)*D10</f>
-        <v>3.0624999999999999E-2</v>
+        <v>4.2500000000000003E-3</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>24</v>
       </c>
@@ -1441,7 +1681,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="1">
-        <v>1.75</v>
+        <v>0.25</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>19</v>
@@ -1456,7 +1696,7 @@
       </c>
       <c r="J8" s="8">
         <f>E2*J6+D9</f>
-        <v>0.74999999999999978</v>
+        <v>0.79999999999999982</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>12</v>
@@ -1469,13 +1709,13 @@
       </c>
       <c r="P8" s="2">
         <f>(J13 * 100)/(ABS(J7) * POWER(10, (I2 / 20)))</f>
-        <v>1.9949999999999999E-2</v>
+        <v>2.0538235294117649E-2</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1498,7 +1738,7 @@
       </c>
       <c r="J9" s="8">
         <f>E2*J7+D9</f>
-        <v>4.25</v>
+        <v>4.2</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>12</v>
@@ -1511,13 +1751,13 @@
       </c>
       <c r="P9" s="2">
         <f>(J14 * 100)/(ABS(J6) * POWER(10, (I2 / 20)))</f>
-        <v>2.0049999999999998E-2</v>
+        <v>2.0638235294117645E-2</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
@@ -1525,7 +1765,7 @@
         <v>11</v>
       </c>
       <c r="D10" s="1">
-        <v>0.01</v>
+        <v>6.8000000000000005E-2</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>36</v>
@@ -1546,7 +1786,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1559,13 +1799,13 @@
       </c>
       <c r="J11" s="2">
         <f>D6 - J7</f>
-        <v>3.4824999999999999</v>
+        <v>3.4830000000000001</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -1578,13 +1818,13 @@
       </c>
       <c r="J12" s="2">
         <f>D6 - J6</f>
-        <v>3.5175000000000001</v>
+        <v>3.5169999999999999</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H13" s="1" t="s">
         <v>43</v>
       </c>
@@ -1593,13 +1833,13 @@
       </c>
       <c r="J13" s="2">
         <f>(J10 + J11) / 2</f>
-        <v>3.49125</v>
+        <v>3.4915000000000003</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H14" s="2" t="s">
         <v>45</v>
       </c>
@@ -1608,7 +1848,7 @@
       </c>
       <c r="J14" s="2">
         <f>(J10 + J12) / 2</f>
-        <v>3.50875</v>
+        <v>3.5084999999999997</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>12</v>
@@ -1628,28 +1868,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F2E2C88-472F-40E6-9BB7-0CE3D1C9A840}">
   <dimension ref="B1:Q10"/>
-  <sheetFormatPr defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="7" width="9.109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="34.44140625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="40.88671875" style="5" customWidth="1"/>
-    <col min="10" max="10" width="25.44140625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" style="5" customWidth="1"/>
-    <col min="12" max="13" width="9.109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="34.44140625" style="5" customWidth="1"/>
-    <col min="15" max="15" width="52.88671875" style="5" customWidth="1"/>
-    <col min="16" max="16" width="17.5546875" style="5" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" style="5" customWidth="1"/>
-    <col min="18" max="16380" width="9.109375" style="5" customWidth="1"/>
-    <col min="16381" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="58.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="7" width="9.140625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="34.42578125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="40.85546875" style="5" customWidth="1"/>
+    <col min="10" max="10" width="25.42578125" style="5" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="9.140625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="34.42578125" style="5" customWidth="1"/>
+    <col min="15" max="15" width="52.85546875" style="5" customWidth="1"/>
+    <col min="16" max="16" width="17.5703125" style="5" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" style="5" customWidth="1"/>
+    <col min="18" max="16380" width="9.140625" style="5" customWidth="1"/>
+    <col min="16381" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1667,7 +1907,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>47</v>
       </c>
@@ -1693,7 +1933,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="10" t="s">
         <v>6</v>
       </c>
@@ -1735,7 +1975,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>51</v>
       </c>
@@ -1772,14 +2012,14 @@
         <v>55</v>
       </c>
       <c r="P5" s="14">
-        <f>POWER(J7, 2) * (D5+D7)</f>
+        <f>POWER(J7,2)*(D5+D7)</f>
         <v>2.3654745406422815E-4</v>
       </c>
       <c r="Q5" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>56</v>
       </c>
@@ -1823,7 +2063,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>62</v>
       </c>
@@ -1858,7 +2098,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>66</v>
       </c>
@@ -1893,7 +2133,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1911,7 +2151,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1938,17 +2178,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD44C968-61FF-4F4E-9D6C-A1C9337DEECD}">
   <dimension ref="B1:Q8"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="58.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1966,7 +2206,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -1992,12 +2232,12 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D3" s="5">
         <v>2.5</v>
@@ -2006,12 +2246,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D4" s="1">
         <v>3.5</v>
@@ -2032,7 +2272,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -2050,7 +2290,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -2068,7 +2308,7 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2086,7 +2326,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -2112,15 +2352,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC3F59B-30C5-40B9-A90E-89A9AC3DA184}">
-  <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S17"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="20" width="16.77734375" style="5" customWidth="1"/>
-    <col min="21" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="20" width="16.7109375" style="5" customWidth="1"/>
+    <col min="21" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
@@ -2140,7 +2380,7 @@
       <c r="R1" s="15"/>
       <c r="S1" s="15"/>
     </row>
-    <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="21" t="s">
         <v>70</v>
       </c>
@@ -2155,13 +2395,13 @@
       <c r="G2" s="21"/>
       <c r="H2" s="10"/>
       <c r="I2" s="21" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="J2" s="21"/>
       <c r="K2" s="21"/>
       <c r="L2" s="21"/>
     </row>
-    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="10" t="s">
         <v>69</v>
       </c>
@@ -2189,15 +2429,15 @@
       </c>
       <c r="L3" s="21"/>
     </row>
-    <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B4" s="1">
-        <v>4.25</v>
+        <v>4.2</v>
       </c>
       <c r="C4" s="1">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="D4" s="1">
         <v>3.5</v>
@@ -2213,55 +2453,61 @@
       </c>
       <c r="H4" s="10"/>
       <c r="I4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="L4" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="1">
-        <v>4.2569999999999997</v>
-      </c>
-      <c r="C5" s="1">
-        <v>0.74299999999999999</v>
-      </c>
-      <c r="D5" s="1">
-        <v>3.4060000000000001</v>
-      </c>
-      <c r="E5" s="1">
+      <c r="B5" s="23">
+        <f>5*C11/(B11+C11)</f>
+        <v>4.2572463768115938</v>
+      </c>
+      <c r="C5" s="23">
+        <f>5*E11/(D11+E11)</f>
+        <v>0.74275362318840576</v>
+      </c>
+      <c r="D5" s="23">
+        <f>5*G11/(F11+G11)</f>
+        <v>3.5652173913043477</v>
+      </c>
+      <c r="E5" s="23">
+        <f>5*I11/(H11+I11)</f>
         <v>2.5</v>
       </c>
-      <c r="F5" s="1">
-        <v>4.468</v>
-      </c>
-      <c r="G5" s="1">
-        <v>0.53200000000000003</v>
+      <c r="F5" s="23">
+        <f>5*K11/(J11+K11)</f>
+        <v>4.4676806083650185</v>
+      </c>
+      <c r="G5" s="23">
+        <f>5*M11/(L11+M11)</f>
+        <v>0.53231939163498099</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1" t="s">
         <v>50</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>50</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -2279,7 +2525,7 @@
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
     </row>
-    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2299,7 +2545,7 @@
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
     </row>
-    <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="21" t="s">
         <v>70</v>
       </c>
@@ -2325,7 +2571,7 @@
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
     </row>
-    <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="21" t="s">
         <v>69</v>
       </c>
@@ -2351,7 +2597,7 @@
       </c>
       <c r="M9" s="21"/>
     </row>
-    <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>56</v>
       </c>
@@ -2389,49 +2635,134 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="22">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C11" s="23">
+        <v>47</v>
+      </c>
+      <c r="D11" s="23">
+        <v>47</v>
+      </c>
+      <c r="E11" s="23">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="F11" s="22">
+        <v>3.3</v>
+      </c>
+      <c r="G11" s="23">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="H11" s="23">
+        <v>47</v>
+      </c>
+      <c r="I11" s="23">
+        <v>47</v>
+      </c>
+      <c r="J11" s="22">
+        <v>5.6</v>
+      </c>
+      <c r="K11" s="23">
+        <v>47</v>
+      </c>
+      <c r="L11" s="23">
+        <v>47</v>
+      </c>
+      <c r="M11" s="23">
+        <v>5.6</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" s="21"/>
+    </row>
+    <row r="14" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="5">
+        <f>(C5-2.5)/(100*0.068)</f>
+        <v>-0.25841858482523444</v>
+      </c>
+      <c r="C15" s="5">
+        <f>(B5-2.5)/(100*0.068)</f>
+        <v>0.25841858482523433</v>
+      </c>
+      <c r="D15" s="24">
+        <f>E5</f>
+        <v>2.5</v>
+      </c>
+      <c r="E15" s="24">
+        <f>D5</f>
+        <v>3.5652173913043477</v>
+      </c>
+      <c r="F15" s="5">
+        <f>10000*G5/(5-G5)</f>
+        <v>1191.4893617021276</v>
+      </c>
+      <c r="G15" s="5">
+        <f>10000*F5/(5-F5)</f>
+        <v>83928.571428571333</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F16" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="6:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F17" s="5">
         <v>77</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>83</v>
+      <c r="G17" s="5">
+        <v>-10.1</v>
+      </c>
+      <c r="H17" s="25" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="18">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>
@@ -2455,19 +2786,19 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DDA2E54-9BDB-4BF6-80B7-49457B01E1DD}">
-  <dimension ref="B1:Q8"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DDA2E54-9BDB-4BF6-80B7-49457B01E1DD}">
+  <dimension ref="B1:Q11"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.42578125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2485,7 +2816,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2511,33 +2842,33 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="73.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D3" s="5">
         <v>16000</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D4" s="5">
         <f>D3 / 2</f>
         <v>8000</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -2552,7 +2883,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>56</v>
       </c>
@@ -2578,19 +2909,19 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D6" s="1">
         <f>1 / (2 * PI() * D5 *D4)</f>
         <v>4.232844231167429E-9</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -2605,7 +2936,7 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2623,11 +2954,19 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>9</v>
+      </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -2641,26 +2980,66 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="5">
+        <v>4700</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="5">
+        <f>0.0000000047</f>
+        <v>4.6999999999999999E-9</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D11" s="5">
+        <f>1/(2*PI()*D9*D10)</f>
+        <v>7204.8412445403055</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBF5C97-B701-49E8-8D17-B57E480030E6}">
-  <dimension ref="B1:Q8"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBF5C97-B701-49E8-8D17-B57E480030E6}">
+  <dimension ref="B1:Q15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.42578125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2678,7 +3057,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2704,7 +3083,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="73.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>56</v>
       </c>
@@ -2716,13 +3095,13 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>76</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1">
-        <v>47000</v>
+        <v>10000</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>36</v>
@@ -2740,13 +3119,13 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="16">
-        <v>10000</v>
+        <v>470000</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>36</v>
@@ -2764,7 +3143,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -2788,18 +3167,18 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="1" t="s">
-        <v>96</v>
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="26" t="s">
+        <v>108</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D7" s="16">
-        <v>9.9999999999999995E-7</v>
+        <v>1E-10</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -2814,11 +3193,20 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8" s="16">
+        <f>D7*1.05</f>
+        <v>1.0500000000000001E-10</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>90</v>
+      </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -2832,9 +3220,79 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" s="27">
+        <f>1/(-2*LN(1/3)*D5*D7)</f>
+        <v>9683.3960279450785</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" s="27">
+        <f>1/(-2*LN(1/3)*D5*D8)</f>
+        <v>9222.2819313762629</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D13" s="16">
+        <v>2000000</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="28">
+        <f>D13/D10</f>
+        <v>206.53911026960463</v>
+      </c>
+    </row>
+    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" s="28">
+        <f>D13/D11</f>
+        <v>216.86606578308491</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added new section to temp sensor sheet, calculates detected temp based on a preferred output voltage
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/ctra157_uoa_auckland_ac_nz/Documents/Documents/GitHub/311/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{F35946E6-0E9C-4E36-9C30-D1AE339D86FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66C118AF-E92A-435A-AB54-0F63D7562F70}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF83167-29AA-4D2C-9F19-8FB03B27FB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
@@ -91,7 +91,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>ctra157:</t>
         </r>
@@ -100,7 +100,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Assumes R1=R2.</t>
@@ -115,7 +115,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>ctra157:</t>
         </r>
@@ -124,7 +124,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 Assumes R1=R2.</t>
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="127">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -531,6 +531,33 @@
   <si>
     <t>TC frequency / f_0</t>
   </si>
+  <si>
+    <t>V_high</t>
+  </si>
+  <si>
+    <t>R_25</t>
+  </si>
+  <si>
+    <t>R_t / R_25</t>
+  </si>
+  <si>
+    <t>(-V_high * R1) / (R_25 * (V_high - Vcc))</t>
+  </si>
+  <si>
+    <t>Corresponding temp range: -15°C to -20°C</t>
+  </si>
+  <si>
+    <t>Supply voltage</t>
+  </si>
+  <si>
+    <t>Thermistor resistance at 25°C</t>
+  </si>
+  <si>
+    <t>Sensor max output voltage</t>
+  </si>
+  <si>
+    <t>Here the snesor output voltage is chosen, then the temperature is determined. Kind of reverse of the above.</t>
+  </si>
 </sst>
 </file>
 
@@ -541,7 +568,7 @@
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -653,19 +680,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -693,7 +707,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -743,21 +757,6 @@
     <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -778,6 +777,27 @@
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -808,8 +828,8 @@
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>103910</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>443627</xdr:rowOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>281</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -863,8 +883,8 @@
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1790700</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1474,26 +1494,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:Q14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="67.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="38.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" style="2" customWidth="1"/>
-    <col min="5" max="7" width="9.140625" style="2"/>
-    <col min="8" max="9" width="38.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" style="2" customWidth="1"/>
-    <col min="11" max="13" width="9.140625" style="2"/>
-    <col min="14" max="14" width="47.7109375" style="2" customWidth="1"/>
-    <col min="15" max="15" width="76.140625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="18.7109375" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="40.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="67.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="38.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" style="2" customWidth="1"/>
+    <col min="5" max="7" width="9.109375" style="2"/>
+    <col min="8" max="9" width="38.6640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="2" customWidth="1"/>
+    <col min="11" max="13" width="9.109375" style="2"/>
+    <col min="14" max="14" width="47.6640625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="76.109375" style="2" customWidth="1"/>
+    <col min="16" max="16" width="18.6640625" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="7"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -1517,7 +1537,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1529,27 +1549,27 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
+    <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="N4" s="18" t="s">
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="N4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-    </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O4" s="25"/>
+      <c r="P4" s="25"/>
+      <c r="Q4" s="25"/>
+    </row>
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
@@ -1589,7 +1609,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1612,7 +1632,7 @@
       </c>
       <c r="J6" s="1">
         <f>D7*D10</f>
-        <v>-1.7000000000000001E-2</v>
+        <v>-1.4999999999999999E-2</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>12</v>
@@ -1625,13 +1645,13 @@
       </c>
       <c r="P6" s="2">
         <f>POWER(D7,2)*D10</f>
-        <v>4.2500000000000003E-3</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
@@ -1639,7 +1659,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="1">
-        <v>-0.25</v>
+        <v>-1.5</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>19</v>
@@ -1654,7 +1674,7 @@
       </c>
       <c r="J7" s="1">
         <f>D8*D10</f>
-        <v>1.7000000000000001E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>12</v>
@@ -1667,13 +1687,13 @@
       </c>
       <c r="P7" s="2">
         <f>POWER(D8,2)*D10</f>
-        <v>4.2500000000000003E-3</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>24</v>
       </c>
@@ -1681,7 +1701,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="1">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>19</v>
@@ -1696,7 +1716,7 @@
       </c>
       <c r="J8" s="8">
         <f>E2*J6+D9</f>
-        <v>0.79999999999999982</v>
+        <v>1</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>12</v>
@@ -1709,13 +1729,13 @@
       </c>
       <c r="P8" s="2">
         <f>(J13 * 100)/(ABS(J7) * POWER(10, (I2 / 20)))</f>
-        <v>2.0538235294117649E-2</v>
+        <v>2.3283333333333333E-2</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1738,7 +1758,7 @@
       </c>
       <c r="J9" s="8">
         <f>E2*J7+D9</f>
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>12</v>
@@ -1751,13 +1771,13 @@
       </c>
       <c r="P9" s="2">
         <f>(J14 * 100)/(ABS(J6) * POWER(10, (I2 / 20)))</f>
-        <v>2.0638235294117645E-2</v>
+        <v>2.3383333333333332E-2</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
@@ -1765,7 +1785,7 @@
         <v>11</v>
       </c>
       <c r="D10" s="1">
-        <v>6.8000000000000005E-2</v>
+        <v>0.01</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>36</v>
@@ -1786,7 +1806,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1799,13 +1819,13 @@
       </c>
       <c r="J11" s="2">
         <f>D6 - J7</f>
-        <v>3.4830000000000001</v>
+        <v>3.4849999999999999</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -1818,13 +1838,13 @@
       </c>
       <c r="J12" s="2">
         <f>D6 - J6</f>
-        <v>3.5169999999999999</v>
+        <v>3.5150000000000001</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H13" s="1" t="s">
         <v>43</v>
       </c>
@@ -1833,13 +1853,13 @@
       </c>
       <c r="J13" s="2">
         <f>(J10 + J11) / 2</f>
-        <v>3.4915000000000003</v>
+        <v>3.4924999999999997</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H14" s="2" t="s">
         <v>45</v>
       </c>
@@ -1848,7 +1868,7 @@
       </c>
       <c r="J14" s="2">
         <f>(J10 + J12) / 2</f>
-        <v>3.5084999999999997</v>
+        <v>3.5075000000000003</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>12</v>
@@ -1867,29 +1887,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F2E2C88-472F-40E6-9BB7-0CE3D1C9A840}">
-  <dimension ref="B1:Q10"/>
-  <sheetFormatPr defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:Q17"/>
+  <sheetFormatPr defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="58.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
-    <col min="6" max="7" width="9.140625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="34.42578125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="40.85546875" style="5" customWidth="1"/>
-    <col min="10" max="10" width="25.42578125" style="5" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" style="5" customWidth="1"/>
-    <col min="12" max="13" width="9.140625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="34.42578125" style="5" customWidth="1"/>
-    <col min="15" max="15" width="52.85546875" style="5" customWidth="1"/>
-    <col min="16" max="16" width="17.5703125" style="5" customWidth="1"/>
-    <col min="17" max="17" width="9.7109375" style="5" customWidth="1"/>
-    <col min="18" max="16380" width="9.140625" style="5" customWidth="1"/>
-    <col min="16381" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="7" width="9.109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="34.44140625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="40.88671875" style="5" customWidth="1"/>
+    <col min="10" max="10" width="25.44140625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" style="5" customWidth="1"/>
+    <col min="12" max="13" width="9.109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="34.44140625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="52.88671875" style="5" customWidth="1"/>
+    <col min="16" max="16" width="17.5546875" style="5" customWidth="1"/>
+    <col min="17" max="17" width="34.44140625" style="5" customWidth="1"/>
+    <col min="18" max="16380" width="9.109375" style="5" customWidth="1"/>
+    <col min="16381" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1907,7 +1927,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>47</v>
       </c>
@@ -1933,7 +1953,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
         <v>6</v>
       </c>
@@ -1975,7 +1995,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>51</v>
       </c>
@@ -2019,7 +2039,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>56</v>
       </c>
@@ -2063,7 +2083,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>62</v>
       </c>
@@ -2098,7 +2118,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>66</v>
       </c>
@@ -2133,7 +2153,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -2151,7 +2171,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -2169,7 +2189,101 @@
       <c r="P10" s="10"/>
       <c r="Q10" s="10"/>
     </row>
+    <row r="11" spans="2:17" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N11" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="O11" s="30"/>
+      <c r="P11" s="30"/>
+      <c r="Q11" s="30"/>
+    </row>
+    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N12" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="O12" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P12" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q12" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P13" s="5">
+        <v>5</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="P14" s="5">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N15" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="P15" s="5">
+        <v>10000</v>
+      </c>
+      <c r="Q15" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="2:17" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I16" s="1"/>
+      <c r="N16" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="P16" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="14:17" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N17" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="O17" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="P17" s="5">
+        <f>(-1*P16*P14)/(P15*(P16-P13))</f>
+        <v>9</v>
+      </c>
+      <c r="Q17" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="N11:Q11"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2178,17 +2292,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD44C968-61FF-4F4E-9D6C-A1C9337DEECD}">
   <dimension ref="B1:Q8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="58.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2206,7 +2320,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2232,7 +2346,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>92</v>
       </c>
@@ -2246,7 +2360,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>94</v>
       </c>
@@ -2272,7 +2386,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -2290,7 +2404,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -2308,7 +2422,7 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2326,7 +2440,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -2353,14 +2467,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC3F59B-30C5-40B9-A90E-89A9AC3DA184}">
   <dimension ref="A1:S17"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="20" width="16.7109375" style="5" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="20" width="16.6640625" style="5" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
@@ -2380,28 +2494,28 @@
       <c r="R1" s="15"/>
       <c r="S1" s="15"/>
     </row>
-    <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="21" t="s">
+    <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21" t="s">
+      <c r="C2" s="28"/>
+      <c r="D2" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21" t="s">
+      <c r="E2" s="28"/>
+      <c r="F2" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="21"/>
+      <c r="G2" s="28"/>
       <c r="H2" s="10"/>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-    </row>
-    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+    </row>
+    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="10" t="s">
         <v>69</v>
       </c>
@@ -2420,16 +2534,16 @@
       <c r="G3" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21" t="s">
+      <c r="J3" s="28"/>
+      <c r="K3" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="L3" s="21"/>
-    </row>
-    <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L3" s="28"/>
+    </row>
+    <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>74</v>
       </c>
@@ -2465,31 +2579,31 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="18">
         <f>5*C11/(B11+C11)</f>
         <v>4.2572463768115938</v>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="18">
         <f>5*E11/(D11+E11)</f>
         <v>0.74275362318840576</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="18">
         <f>5*G11/(F11+G11)</f>
         <v>3.5652173913043477</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="18">
         <f>5*I11/(H11+I11)</f>
         <v>2.5</v>
       </c>
-      <c r="F5" s="23">
+      <c r="F5" s="18">
         <f>5*K11/(J11+K11)</f>
         <v>4.4676806083650185</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="18">
         <f>5*M11/(L11+M11)</f>
         <v>0.53231939163498099</v>
       </c>
@@ -2507,7 +2621,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -2525,7 +2639,7 @@
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
     </row>
-    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2545,25 +2659,25 @@
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
     </row>
-    <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="21" t="s">
+    <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21" t="s">
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21" t="s">
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
+      <c r="K8" s="28"/>
+      <c r="L8" s="28"/>
+      <c r="M8" s="28"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -2571,33 +2685,33 @@
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
     </row>
-    <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="21" t="s">
+    <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21" t="s">
+      <c r="C9" s="28"/>
+      <c r="D9" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21" t="s">
+      <c r="E9" s="28"/>
+      <c r="F9" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21" t="s">
+      <c r="G9" s="28"/>
+      <c r="H9" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="I9" s="21"/>
-      <c r="J9" s="21" t="s">
+      <c r="I9" s="28"/>
+      <c r="J9" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="K9" s="21"/>
-      <c r="L9" s="21" t="s">
+      <c r="K9" s="28"/>
+      <c r="L9" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="M9" s="21"/>
-    </row>
-    <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M9" s="28"/>
+    </row>
+    <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>56</v>
       </c>
@@ -2635,65 +2749,65 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="17">
         <v>8.1999999999999993</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="18">
         <v>47</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="18">
         <v>47</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="18">
         <v>8.1999999999999993</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="17">
         <v>3.3</v>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="18">
         <v>8.1999999999999993</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="18">
         <v>47</v>
       </c>
-      <c r="I11" s="23">
+      <c r="I11" s="18">
         <v>47</v>
       </c>
-      <c r="J11" s="22">
+      <c r="J11" s="17">
         <v>5.6</v>
       </c>
-      <c r="K11" s="23">
+      <c r="K11" s="18">
         <v>47</v>
       </c>
-      <c r="L11" s="23">
+      <c r="L11" s="18">
         <v>47</v>
       </c>
-      <c r="M11" s="23">
+      <c r="M11" s="18">
         <v>5.6</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="21" t="s">
+    <row r="13" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21" t="s">
+      <c r="C13" s="28"/>
+      <c r="D13" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21" t="s">
+      <c r="E13" s="28"/>
+      <c r="F13" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="G13" s="21"/>
-    </row>
-    <row r="14" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="28"/>
+    </row>
+    <row r="14" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>99</v>
       </c>
@@ -2713,7 +2827,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5">
         <f>(C5-2.5)/(100*0.068)</f>
         <v>-0.25841858482523444</v>
@@ -2722,11 +2836,11 @@
         <f>(B5-2.5)/(100*0.068)</f>
         <v>0.25841858482523433</v>
       </c>
-      <c r="D15" s="24">
+      <c r="D15" s="19">
         <f>E5</f>
         <v>2.5</v>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="19">
         <f>D5</f>
         <v>3.5652173913043477</v>
       </c>
@@ -2739,7 +2853,7 @@
         <v>83928.571428571333</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F16" s="1" t="s">
         <v>105</v>
       </c>
@@ -2747,25 +2861,22 @@
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="6:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="6:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F17" s="5">
         <v>77</v>
       </c>
       <c r="G17" s="5">
         <v>-10.1</v>
       </c>
-      <c r="H17" s="25" t="s">
+      <c r="H17" s="20" t="s">
         <v>107</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:L3"/>
     <mergeCell ref="J8:M8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B8:E8"/>
@@ -2775,9 +2886,12 @@
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="L9:M9"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2788,17 +2902,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DDA2E54-9BDB-4BF6-80B7-49457B01E1DD}">
   <dimension ref="B1:Q11"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="34.42578125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="52.85546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2816,7 +2930,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2842,7 +2956,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="73.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>85</v>
       </c>
@@ -2856,7 +2970,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>88</v>
       </c>
@@ -2883,7 +2997,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>56</v>
       </c>
@@ -2909,7 +3023,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>83</v>
       </c>
@@ -2936,7 +3050,7 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2954,7 +3068,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="10" t="s">
         <v>96</v>
       </c>
@@ -2980,7 +3094,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>56</v>
       </c>
@@ -2991,7 +3105,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>83</v>
       </c>
@@ -3003,7 +3117,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>88</v>
       </c>
@@ -3029,17 +3143,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBF5C97-B701-49E8-8D17-B57E480030E6}">
   <dimension ref="B1:Q15"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="34.42578125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="52.85546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3057,7 +3171,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -3083,7 +3197,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="73.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>56</v>
       </c>
@@ -3095,7 +3209,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>76</v>
       </c>
@@ -3119,7 +3233,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>77</v>
       </c>
@@ -3143,7 +3257,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -3167,8 +3281,8 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="26" t="s">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="21" t="s">
         <v>108</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -3193,8 +3307,8 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="26" t="s">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="21" t="s">
         <v>109</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -3220,14 +3334,14 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>110</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D10" s="27">
+      <c r="D10" s="22">
         <f>1/(-2*LN(1/3)*D5*D7)</f>
         <v>9683.3960279450785</v>
       </c>
@@ -3235,14 +3349,14 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>111</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D11" s="27">
+      <c r="D11" s="22">
         <f>1/(-2*LN(1/3)*D5*D8)</f>
         <v>9222.2819313762629</v>
       </c>
@@ -3250,7 +3364,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>113</v>
       </c>
@@ -3264,26 +3378,26 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="26" t="s">
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="21" t="s">
         <v>114</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="23">
         <f>D13/D10</f>
         <v>206.53911026960463</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="26" t="s">
+    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="21" t="s">
         <v>115</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="23">
         <f>D13/D11</f>
         <v>216.86606578308491</v>
       </c>

</xml_diff>